<commit_message>
Actualización HV posdoc para UEB
</commit_message>
<xml_diff>
--- a/PDF/data/experiencia_docente.xlsx
+++ b/PDF/data/experiencia_docente.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">why</t>
   </si>
   <si>
-    <t xml:space="preserve">Posdoctorado</t>
+    <t xml:space="preserve">Estancia Posdoctoral</t>
   </si>
   <si>
     <t xml:space="preserve">Desde 2023</t>

</xml_diff>

<commit_message>
Creamos HV académica corta, agregamos link a microsotio en todas las HVs, correcciones de errores menores, y artículo pedagogías de la crueldad publicado
</commit_message>
<xml_diff>
--- a/PDF/data/experiencia_docente.xlsx
+++ b/PDF/data/experiencia_docente.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t xml:space="preserve">what</t>
   </si>
@@ -37,16 +37,28 @@
     <t xml:space="preserve">why</t>
   </si>
   <si>
+    <t xml:space="preserve">Docente Investigadora – Facultad de Psicología</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desde 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidad El Bosque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profesora Asociada</t>
+  </si>
+  <si>
     <t xml:space="preserve">Estancia Posdoctoral</t>
   </si>
   <si>
-    <t xml:space="preserve">Desde 2023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asociación Red de Mujeres Víctimas y Profesionales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bogotá, Colombia</t>
+    <t xml:space="preserve">2023 – 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asociación Red de Mujeres Víctimas y Profesionales – Minciencias</t>
   </si>
   <si>
     <t xml:space="preserve">\textbf{Proyecto: } La necesidad de generar procesos de reparación social a las mujeres víctimas y sobrevivientes de violencias sexuales en el marco del conflicto armado desde el quehacer periodístico. Diversas propuestas de tratamiento según contextos</t>
@@ -405,52 +417,60 @@
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="E3" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -459,7 +479,7 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -468,7 +488,7 @@
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -477,7 +497,7 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -486,7 +506,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -495,7 +515,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -504,7 +524,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -513,7 +533,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -521,9 +541,18 @@
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="E13" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Agregar capítulo de libro Violencia sexual y reparación
</commit_message>
<xml_diff>
--- a/PDF/data/experiencia_docente.xlsx
+++ b/PDF/data/experiencia_docente.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">why</t>
   </si>
   <si>
-    <t xml:space="preserve">Docente Investigadora – Facultad de Psicología</t>
+    <t xml:space="preserve">Docente Investigadora – Facultad de Psicología y Centro de Diversidad, Equidad e Inclusión</t>
   </si>
   <si>
     <t xml:space="preserve">Desde 2026</t>
@@ -387,7 +387,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E1048576"/>
-  <sheetFormatPr defaultColWidth="8.890625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.89453125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.34"/>

</xml_diff>